<commit_message>
Map zoom/pan with floor plan zoom/pan.
</commit_message>
<xml_diff>
--- a/data/exhibitors.xlsx
+++ b/data/exhibitors.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="128">
   <si>
     <t>name</t>
   </si>
@@ -240,6 +240,174 @@
   </si>
   <si>
     <t>Wayne County Department of Social Services</t>
+  </si>
+  <si>
+    <t>Brian Manktelow</t>
+  </si>
+  <si>
+    <t>Supporting economic growth, reducing state mandates, and protecting local resources</t>
+  </si>
+  <si>
+    <t>Council on Alcoholism and Addiction</t>
+  </si>
+  <si>
+    <t>Empowering Lives, Transforming Communities</t>
+  </si>
+  <si>
+    <t>Finger Lakes Area Intergroup</t>
+  </si>
+  <si>
+    <t>Alcohol and addiction services</t>
+  </si>
+  <si>
+    <t>Finger Lakes Community Action</t>
+  </si>
+  <si>
+    <t>Helping people, and changing lives</t>
+  </si>
+  <si>
+    <t>Grange</t>
+  </si>
+  <si>
+    <t>In essentials, unity; in non-essentials, liberty; in all things, charity</t>
+  </si>
+  <si>
+    <t>NY Army National Guard</t>
+  </si>
+  <si>
+    <t>Always Ready, Always There</t>
+  </si>
+  <si>
+    <t>Pal Mac Robotics</t>
+  </si>
+  <si>
+    <t>Designing and building competitive robots, building life skills, and participating in tournaments</t>
+  </si>
+  <si>
+    <t>Palmyra American Legion</t>
+  </si>
+  <si>
+    <t>Veterans Strengthening America</t>
+  </si>
+  <si>
+    <t>S.C.O.P.E.</t>
+  </si>
+  <si>
+    <t>Protect, Restore, and Expand the gun rights of all New Yorkers</t>
+  </si>
+  <si>
+    <t>Model Trains Exhibit</t>
+  </si>
+  <si>
+    <t>Model trains for everyone</t>
+  </si>
+  <si>
+    <t>Wayne County Conservative Party</t>
+  </si>
+  <si>
+    <t>Protecting the taxpayers of New York State</t>
+  </si>
+  <si>
+    <t>Wayne County Democrats</t>
+  </si>
+  <si>
+    <t>To ensure the success of the Democratic Party</t>
+  </si>
+  <si>
+    <t>Wayne County Libraries</t>
+  </si>
+  <si>
+    <t>Community, Connections, Discovery</t>
+  </si>
+  <si>
+    <t>Wayne County Republicans</t>
+  </si>
+  <si>
+    <t>The party of opportunity</t>
+  </si>
+  <si>
+    <t>Wolcott Lions Club</t>
+  </si>
+  <si>
+    <t>Where there's a need, there's a Lion</t>
+  </si>
+  <si>
+    <t>Rochester Regional Health</t>
+  </si>
+  <si>
+    <t>We're Here For It</t>
+  </si>
+  <si>
+    <t>Best In Show Beer Tent</t>
+  </si>
+  <si>
+    <t>Commercial 2</t>
+  </si>
+  <si>
+    <t>Commercial 1</t>
+  </si>
+  <si>
+    <t>Entertainment Alley</t>
+  </si>
+  <si>
+    <t>Cold Beer in Here</t>
+  </si>
+  <si>
+    <t>food</t>
+  </si>
+  <si>
+    <t>Daily 5:00 PM - 11:00 PM</t>
+  </si>
+  <si>
+    <t>food/beer.webp</t>
+  </si>
+  <si>
+    <t>exhibit/rrh.webp</t>
+  </si>
+  <si>
+    <t>exhibit/lions.webp</t>
+  </si>
+  <si>
+    <t>exhibit/republicans.webp</t>
+  </si>
+  <si>
+    <t>exhibit/libraries.webp</t>
+  </si>
+  <si>
+    <t>exhibit/democrats.webp</t>
+  </si>
+  <si>
+    <t>exhibit/conservative.webp</t>
+  </si>
+  <si>
+    <t>exhibit/trains.webp</t>
+  </si>
+  <si>
+    <t>exhibit/scope.webp</t>
+  </si>
+  <si>
+    <t>exhibit/legion.webp</t>
+  </si>
+  <si>
+    <t>exhibit/raiders.webp</t>
+  </si>
+  <si>
+    <t>exhibit/guard.webp</t>
+  </si>
+  <si>
+    <t>exhibit/grange.webp</t>
+  </si>
+  <si>
+    <t>exhibit/action.webp</t>
+  </si>
+  <si>
+    <t>exhibit/intergroup.webp</t>
+  </si>
+  <si>
+    <t>exhibit/addiction.webp</t>
+  </si>
+  <si>
+    <t>exhibit/brian.webp</t>
   </si>
 </sst>
 </file>
@@ -274,7 +442,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -297,17 +465,46 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -590,7 +787,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="33.42578125" customWidth="1"/>
@@ -1108,7 +1305,399 @@
         <v>0</v>
       </c>
     </row>
+    <row r="23" spans="1:7" ht="27" thickBot="1">
+      <c r="A23" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D23" t="s">
+        <v>7</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="F23" t="s">
+        <v>70</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A24" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D24" t="s">
+        <v>7</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F24" t="s">
+        <v>70</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A25" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D25" t="s">
+        <v>7</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="F25" t="s">
+        <v>70</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A26" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D26" t="s">
+        <v>7</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="F26" t="s">
+        <v>70</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="27" thickBot="1">
+      <c r="A27" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D27" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="F27" t="s">
+        <v>70</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A28" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D28" t="s">
+        <v>7</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="F28" t="s">
+        <v>70</v>
+      </c>
+      <c r="G28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="27" thickBot="1">
+      <c r="A29" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D29" t="s">
+        <v>7</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="F29" t="s">
+        <v>70</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A30" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D30" t="s">
+        <v>7</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F30" t="s">
+        <v>70</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="27" thickBot="1">
+      <c r="A31" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D31" t="s">
+        <v>7</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="F31" t="s">
+        <v>70</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A32" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D32" t="s">
+        <v>7</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="F32" t="s">
+        <v>70</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A33" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D33" t="s">
+        <v>7</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="F33" t="s">
+        <v>70</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A34" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D34" t="s">
+        <v>7</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="F34" t="s">
+        <v>70</v>
+      </c>
+      <c r="G34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A35" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D35" t="s">
+        <v>7</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="F35" t="s">
+        <v>70</v>
+      </c>
+      <c r="G35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A36" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D36" t="s">
+        <v>7</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="F36" t="s">
+        <v>70</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A37" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D37" t="s">
+        <v>7</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="F37" t="s">
+        <v>70</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A38" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D38" t="s">
+        <v>7</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="F38" t="s">
+        <v>70</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="27" thickBot="1">
+      <c r="A39" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="G39">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>